<commit_message>
fix: Stock reporting and reconciliation.
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
   <si>
     <t>Product Line</t>
   </si>
@@ -103,6 +103,9 @@
     <t>NMN coffee</t>
   </si>
   <si>
+    <t>893663002425</t>
+  </si>
+  <si>
     <t>print white</t>
   </si>
   <si>
@@ -169,7 +172,10 @@
     <t>893663002609</t>
   </si>
   <si>
-    <t>Detoxilive Capsules</t>
+    <t>Detoxilive Capsules pro</t>
+  </si>
+  <si>
+    <t>487104471401</t>
   </si>
   <si>
     <t>Digestive Health</t>
@@ -286,12 +292,6 @@
     <t>out of stock</t>
   </si>
   <si>
-    <t>SUMA GRAND 1 (Cleanser+Lotion+Toner)</t>
-  </si>
-  <si>
-    <t>SUMA GRAND 2 (Full Set)</t>
-  </si>
-  <si>
     <t>Smart Kids</t>
   </si>
   <si>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>Dr.Ts Toothpaste</t>
+  </si>
+  <si>
+    <t>853913003053</t>
   </si>
   <si>
     <t>print</t>
@@ -351,10 +354,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -388,46 +391,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -443,23 +407,9 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="3"/>
       <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -471,22 +421,7 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -509,14 +444,82 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="15"/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -532,187 +535,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -723,26 +726,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -761,41 +744,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -823,145 +776,195 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -979,6 +982,7 @@
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1240,7 +1244,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="12.6283185840708" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.2477876106195" customWidth="1"/>
@@ -1283,7 +1287,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="2">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2">
         <v>6.5</v>
@@ -1303,7 +1307,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="2">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2">
         <v>6.5</v>
@@ -1323,7 +1327,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D4" s="2">
         <v>6.5</v>
@@ -1343,7 +1347,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="2">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D5" s="2">
         <v>52</v>
@@ -1363,7 +1367,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="2">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D6" s="2">
         <v>99</v>
@@ -1383,7 +1387,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2">
         <v>102</v>
@@ -1423,7 +1427,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="2">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D9" s="2">
         <v>28</v>
@@ -1446,7 +1450,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2">
         <v>79</v>
@@ -1466,7 +1470,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="2">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D11" s="2">
         <v>12.5</v>
@@ -1477,13 +1481,16 @@
       <c r="F11" s="5">
         <v>3375</v>
       </c>
+      <c r="H11" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="I11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="2:8">
       <c r="B12" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" s="2">
         <v>17</v>
@@ -1498,15 +1505,15 @@
         <v>21600</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="2:8">
       <c r="B13" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C13" s="2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D13" s="2">
         <v>112</v>
@@ -1518,15 +1525,15 @@
         <v>20115</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:6">
       <c r="A14" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C14" s="2">
         <v>0</v>
@@ -1543,10 +1550,10 @@
     </row>
     <row r="15" customHeight="1" spans="2:8">
       <c r="B15" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="2">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D15" s="2">
         <v>34.5</v>
@@ -1558,15 +1565,15 @@
         <v>5400</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="2:8">
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" s="2">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="D16" s="2">
         <v>18</v>
@@ -1578,12 +1585,12 @@
         <v>3105</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="2:8">
       <c r="B17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C17" s="2">
         <v>0</v>
@@ -1598,18 +1605,18 @@
         <v>7560</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C18" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D18" s="2">
         <v>11</v>
@@ -1621,15 +1628,15 @@
         <v>2970</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" customHeight="1" spans="2:8">
       <c r="B19" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C19" s="2">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="D19" s="2">
         <v>22</v>
@@ -1641,15 +1648,15 @@
         <v>3375</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" customHeight="1" spans="2:8">
       <c r="B20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C20" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D20" s="2">
         <v>9</v>
@@ -1661,15 +1668,15 @@
         <v>2430</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="2:8">
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C21" s="2">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D21" s="2">
         <v>15</v>
@@ -1681,35 +1688,38 @@
         <v>2700</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" customHeight="1" spans="2:6">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" customHeight="1" spans="2:8">
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" s="2">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D22" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E22" s="4">
-        <v>2632.5</v>
+        <v>3510</v>
       </c>
       <c r="F22" s="5">
-        <v>2025</v>
+        <v>2700</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C23" s="2">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D23" s="2">
         <v>22</v>
@@ -1721,15 +1731,15 @@
         <v>3915</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="2:8">
       <c r="B24" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C24" s="2">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="D24" s="2">
         <v>2.4</v>
@@ -1741,15 +1751,15 @@
         <v>1620</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="2:8">
       <c r="B25" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C25" s="2">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D25" s="2">
         <v>15</v>
@@ -1761,15 +1771,15 @@
         <v>4050</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="2:8">
       <c r="B26" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C26" s="2">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D26" s="2">
         <v>17</v>
@@ -1781,15 +1791,15 @@
         <v>2970</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="2:8">
       <c r="B27" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C27" s="2">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="D27" s="2">
         <v>22</v>
@@ -1801,15 +1811,15 @@
         <v>4050</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="2:8">
       <c r="B28" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C28" s="2">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="D28" s="2">
         <v>23</v>
@@ -1821,12 +1831,12 @@
         <v>4050</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="2:8">
       <c r="B29" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C29" s="2">
         <v>0</v>
@@ -1841,18 +1851,18 @@
         <v>7020</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" s="2">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="D30" s="2">
         <v>18</v>
@@ -1864,15 +1874,15 @@
         <v>3240</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="2:8">
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D31" s="2">
         <v>35</v>
@@ -1884,15 +1894,15 @@
         <v>5670</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="2:8">
       <c r="B32" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C32" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2">
         <v>8</v>
@@ -1904,15 +1914,15 @@
         <v>2025</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" customHeight="1" spans="2:8">
       <c r="B33" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C33" s="2">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D33" s="2">
         <v>25</v>
@@ -1924,15 +1934,15 @@
         <v>4050</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" customHeight="1" spans="2:8">
       <c r="B34" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C34" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D34" s="2">
         <v>24.5</v>
@@ -1944,15 +1954,15 @@
         <v>4320</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="2:8">
       <c r="B35" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C35" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D35" s="2">
         <v>28</v>
@@ -1964,15 +1974,15 @@
         <v>5400</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" customHeight="1" spans="2:8">
       <c r="B36" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C36" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D36" s="2">
         <v>15</v>
@@ -1984,15 +1994,15 @@
         <v>2970</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" customHeight="1" spans="2:8">
       <c r="B37" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C37" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D37" s="2">
         <v>19</v>
@@ -2004,15 +2014,15 @@
         <v>3375</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" customHeight="1" spans="2:8">
       <c r="B38" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C38" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D38" s="2">
         <v>19</v>
@@ -2024,15 +2034,15 @@
         <v>3645</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" customHeight="1" spans="2:8">
       <c r="B39" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C39" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D39" s="2">
         <v>13</v>
@@ -2044,12 +2054,12 @@
         <v>2430</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" customHeight="1" spans="2:9">
       <c r="B40" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C40" s="2">
         <v>0</v>
@@ -2064,199 +2074,172 @@
         <v>4590</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" customHeight="1" spans="2:6">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="41" customHeight="1" spans="1:8">
+      <c r="A41" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="B41" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C41" s="2"/>
+        <v>93</v>
+      </c>
+      <c r="C41" s="2">
+        <v>13</v>
+      </c>
       <c r="D41" s="2">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E41" s="4">
-        <v>12987</v>
+        <v>4212</v>
       </c>
       <c r="F41" s="5">
-        <v>9990</v>
-      </c>
-    </row>
-    <row r="42" customHeight="1" spans="2:6">
+        <v>3240</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="42" customHeight="1" spans="2:8">
       <c r="B42" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C42" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="C42" s="2">
+        <v>28</v>
+      </c>
       <c r="D42" s="2">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="E42" s="4">
-        <v>22113</v>
+        <v>4212</v>
       </c>
       <c r="F42" s="5">
-        <v>17010</v>
-      </c>
-    </row>
-    <row r="43" customHeight="1" spans="1:8">
-      <c r="A43" s="2" t="s">
-        <v>92</v>
-      </c>
+        <v>3240</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="43" customHeight="1" spans="2:8">
       <c r="B43" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C43" s="2">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D43" s="2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E43" s="4">
-        <v>4212</v>
+        <v>3510</v>
       </c>
       <c r="F43" s="5">
-        <v>3240</v>
+        <v>2700</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="44" customHeight="1" spans="2:8">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" customHeight="1" spans="1:8">
+      <c r="A44" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="B44" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C44" s="2">
-        <v>28</v>
+        <v>170</v>
       </c>
       <c r="D44" s="2">
-        <v>18</v>
-      </c>
-      <c r="E44" s="4">
-        <v>4212</v>
-      </c>
-      <c r="F44" s="5">
-        <v>3240</v>
+        <v>1</v>
+      </c>
+      <c r="E44" s="2">
+        <v>386.1</v>
+      </c>
+      <c r="F44" s="3">
+        <v>297</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="2:8">
       <c r="B45" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C45" s="2">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D45" s="2">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E45" s="4">
-        <v>3510</v>
+        <v>1930.5</v>
       </c>
       <c r="F45" s="5">
-        <v>2700</v>
+        <v>1485</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="46" customHeight="1" spans="1:8">
-      <c r="A46" s="2" t="s">
-        <v>99</v>
-      </c>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" customHeight="1" spans="2:9">
       <c r="B46" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C46" s="2">
-        <v>207</v>
+        <v>135</v>
       </c>
       <c r="D46" s="2">
-        <v>1</v>
+        <v>2.8</v>
       </c>
       <c r="E46" s="2">
-        <v>386.1</v>
+        <v>965.25</v>
       </c>
       <c r="F46" s="3">
-        <v>297</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>101</v>
+        <v>743</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="2:8">
       <c r="B47" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C47" s="2">
-        <v>19</v>
+        <v>265</v>
       </c>
       <c r="D47" s="2">
-        <v>6</v>
+        <v>2.4</v>
       </c>
       <c r="E47" s="4">
-        <v>1930.5</v>
+        <v>2106</v>
       </c>
       <c r="F47" s="5">
-        <v>1485</v>
+        <v>1620</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="48" customHeight="1" spans="2:9">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="48" customHeight="1" spans="1:6">
+      <c r="A48" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="B48" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C48" s="2">
-        <v>142</v>
-      </c>
-      <c r="D48" s="2">
-        <v>2.8</v>
-      </c>
-      <c r="E48" s="2">
-        <v>965.25</v>
-      </c>
-      <c r="F48" s="3">
-        <v>743</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="49" customHeight="1" spans="2:8">
-      <c r="B49" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C49" s="2">
-        <v>229</v>
-      </c>
-      <c r="D49" s="2">
-        <v>2.4</v>
-      </c>
-      <c r="E49" s="4">
-        <v>2106</v>
-      </c>
-      <c r="F49" s="5">
-        <v>1620</v>
-      </c>
-      <c r="H49" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="50" customHeight="1" spans="1:6">
-      <c r="A50" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C50">
-        <v>70</v>
-      </c>
-      <c r="E50" s="4">
+        <v>110</v>
+      </c>
+      <c r="C48">
+        <v>63</v>
+      </c>
+      <c r="E48" s="4">
         <v>2900</v>
       </c>
-      <c r="F50" s="5">
+      <c r="F48" s="5">
         <v>2900</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update to products table
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t>Product Line</t>
   </si>
@@ -176,6 +176,9 @@
   </si>
   <si>
     <t>487104471401</t>
+  </si>
+  <si>
+    <t>add</t>
   </si>
   <si>
     <t>Digestive Health</t>
@@ -354,10 +357,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -383,6 +386,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -391,7 +417,97 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -407,124 +523,11 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -535,115 +538,169 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -655,67 +712,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -729,17 +732,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -756,8 +753,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -792,17 +789,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -818,156 +804,173 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1287,7 +1290,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="2">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="D2" s="2">
         <v>6.5</v>
@@ -1307,7 +1310,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="2">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="D3" s="2">
         <v>6.5</v>
@@ -1327,7 +1330,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="D4" s="2">
         <v>6.5</v>
@@ -1347,7 +1350,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="2">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="D5" s="2">
         <v>52</v>
@@ -1367,7 +1370,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="2">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="D6" s="2">
         <v>99</v>
@@ -1387,7 +1390,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="2">
         <v>102</v>
@@ -1407,7 +1410,7 @@
         <v>21</v>
       </c>
       <c r="C8" s="2">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D8" s="2">
         <v>24</v>
@@ -1450,7 +1453,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D10" s="2">
         <v>79</v>
@@ -1470,7 +1473,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2">
         <v>12.5</v>
@@ -1493,7 +1496,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12" s="2">
         <v>128</v>
@@ -1553,7 +1556,7 @@
         <v>37</v>
       </c>
       <c r="C15" s="2">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D15" s="2">
         <v>34.5</v>
@@ -1573,7 +1576,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="2">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2">
         <v>18</v>
@@ -1616,7 +1619,7 @@
         <v>44</v>
       </c>
       <c r="C18" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" s="2">
         <v>11</v>
@@ -1636,7 +1639,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="2">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D19" s="2">
         <v>22</v>
@@ -1656,7 +1659,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="2">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D20" s="2">
         <v>9</v>
@@ -1676,7 +1679,7 @@
         <v>50</v>
       </c>
       <c r="C21" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D21" s="2">
         <v>15</v>
@@ -1691,12 +1694,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="2:8">
+    <row r="22" customHeight="1" spans="2:9">
       <c r="B22" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="2">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D22" s="2">
         <v>15</v>
@@ -1710,16 +1713,19 @@
       <c r="H22" s="7" t="s">
         <v>53</v>
       </c>
+      <c r="I22" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="23" customHeight="1" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D23" s="2">
         <v>22</v>
@@ -1731,15 +1737,15 @@
         <v>3915</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="2:8">
       <c r="B24" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C24" s="2">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="D24" s="2">
         <v>2.4</v>
@@ -1751,12 +1757,12 @@
         <v>1620</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="2:8">
       <c r="B25" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2">
         <v>25</v>
@@ -1771,15 +1777,15 @@
         <v>4050</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="2:8">
       <c r="B26" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C26" s="2">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D26" s="2">
         <v>17</v>
@@ -1791,15 +1797,15 @@
         <v>2970</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="2:8">
       <c r="B27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="2">
         <v>63</v>
-      </c>
-      <c r="C27" s="2">
-        <v>39</v>
       </c>
       <c r="D27" s="2">
         <v>22</v>
@@ -1811,15 +1817,15 @@
         <v>4050</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="2:8">
       <c r="B28" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="D28" s="2">
         <v>23</v>
@@ -1831,12 +1837,12 @@
         <v>4050</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="2:8">
       <c r="B29" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C29" s="2">
         <v>0</v>
@@ -1851,18 +1857,18 @@
         <v>7020</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="D30" s="2">
         <v>18</v>
@@ -1874,15 +1880,15 @@
         <v>3240</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="2:8">
       <c r="B31" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C31" s="2">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D31" s="2">
         <v>35</v>
@@ -1894,15 +1900,15 @@
         <v>5670</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="2:8">
       <c r="B32" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C32" s="2">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D32" s="2">
         <v>8</v>
@@ -1914,15 +1920,15 @@
         <v>2025</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" customHeight="1" spans="2:8">
       <c r="B33" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C33" s="2">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D33" s="2">
         <v>25</v>
@@ -1934,15 +1940,15 @@
         <v>4050</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" customHeight="1" spans="2:8">
       <c r="B34" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C34" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D34" s="2">
         <v>24.5</v>
@@ -1954,12 +1960,12 @@
         <v>4320</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="2:8">
       <c r="B35" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C35" s="2">
         <v>19</v>
@@ -1974,15 +1980,15 @@
         <v>5400</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" customHeight="1" spans="2:8">
       <c r="B36" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C36" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D36" s="2">
         <v>15</v>
@@ -1994,12 +2000,12 @@
         <v>2970</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" customHeight="1" spans="2:8">
       <c r="B37" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C37" s="2">
         <v>0</v>
@@ -2014,15 +2020,15 @@
         <v>3375</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" customHeight="1" spans="2:8">
       <c r="B38" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D38" s="2">
         <v>19</v>
@@ -2034,15 +2040,15 @@
         <v>3645</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" customHeight="1" spans="2:8">
       <c r="B39" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C39" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D39" s="2">
         <v>13</v>
@@ -2054,12 +2060,12 @@
         <v>2430</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" customHeight="1" spans="2:9">
       <c r="B40" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" s="2">
         <v>0</v>
@@ -2074,15 +2080,15 @@
         <v>4590</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41" customHeight="1" spans="1:8">
       <c r="A41" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C41" s="2">
         <v>13</v>
@@ -2097,12 +2103,12 @@
         <v>3240</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" customHeight="1" spans="2:8">
       <c r="B42" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C42" s="2">
         <v>28</v>
@@ -2117,15 +2123,15 @@
         <v>3240</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" customHeight="1" spans="2:8">
       <c r="B43" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C43" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D43" s="2">
         <v>15</v>
@@ -2137,18 +2143,18 @@
         <v>2700</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" customHeight="1" spans="1:8">
       <c r="A44" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C44" s="2">
-        <v>170</v>
+        <v>259</v>
       </c>
       <c r="D44" s="2">
         <v>1</v>
@@ -2160,15 +2166,15 @@
         <v>297</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="2:8">
       <c r="B45" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C45" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D45" s="2">
         <v>6</v>
@@ -2180,15 +2186,15 @@
         <v>1485</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" customHeight="1" spans="2:9">
       <c r="B46" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C46" s="2">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="D46" s="2">
         <v>2.8</v>
@@ -2200,18 +2206,18 @@
         <v>743</v>
       </c>
       <c r="H46" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="2:8">
       <c r="B47" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C47" s="2">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="D47" s="2">
         <v>2.4</v>
@@ -2223,18 +2229,18 @@
         <v>1620</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" customHeight="1" spans="1:6">
       <c r="A48" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C48">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E48" s="4">
         <v>2900</v>

</xml_diff>

<commit_message>
fix: Stock report reconsiliation and product inventory baseline
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -357,9 +357,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
@@ -378,9 +378,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -394,9 +416,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -410,29 +431,29 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF3F3F76"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -447,18 +468,33 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -478,56 +514,20 @@
     </font>
     <font>
       <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -538,19 +538,109 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -562,13 +652,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -580,90 +706,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -671,54 +719,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -741,24 +741,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -770,36 +752,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -821,6 +773,30 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -829,151 +805,175 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2111,7 +2111,7 @@
         <v>96</v>
       </c>
       <c r="C42" s="2">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D42" s="2">
         <v>18</v>

</xml_diff>

<commit_message>
Update to products excel
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -349,7 +349,7 @@
     <t>Registration</t>
   </si>
   <si>
-    <t>Registration Fee</t>
+    <t>Registration Kit</t>
   </si>
 </sst>
 </file>
@@ -357,10 +357,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -373,6 +373,22 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -393,8 +409,38 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -408,8 +454,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="13"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -417,21 +486,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -444,16 +499,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -467,24 +514,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -492,38 +523,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -538,187 +538,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -741,6 +741,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -752,56 +761,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -829,151 +788,192 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1310,7 +1310,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="2">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D3" s="2">
         <v>6.5</v>
@@ -1330,7 +1330,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D4" s="2">
         <v>6.5</v>
@@ -1350,7 +1350,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="2">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="D5" s="2">
         <v>52</v>
@@ -1370,7 +1370,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="2">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D6" s="2">
         <v>99</v>
@@ -1390,7 +1390,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2">
         <v>102</v>
@@ -1410,7 +1410,7 @@
         <v>21</v>
       </c>
       <c r="C8" s="2">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2">
         <v>24</v>
@@ -1430,7 +1430,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="2">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2">
         <v>28</v>
@@ -1453,7 +1453,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10" s="2">
         <v>79</v>
@@ -1473,7 +1473,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="2">
         <v>12.5</v>
@@ -1496,7 +1496,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" s="2">
         <v>128</v>
@@ -1556,7 +1556,7 @@
         <v>37</v>
       </c>
       <c r="C15" s="2">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D15" s="2">
         <v>34.5</v>
@@ -1576,7 +1576,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="2">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D16" s="2">
         <v>18</v>
@@ -1619,7 +1619,7 @@
         <v>44</v>
       </c>
       <c r="C18" s="2">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D18" s="2">
         <v>11</v>
@@ -1639,7 +1639,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="2">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D19" s="2">
         <v>22</v>
@@ -1659,7 +1659,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="2">
         <v>9</v>
@@ -1679,7 +1679,7 @@
         <v>50</v>
       </c>
       <c r="C21" s="2">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D21" s="2">
         <v>15</v>
@@ -1725,7 +1725,7 @@
         <v>56</v>
       </c>
       <c r="C23" s="2">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D23" s="2">
         <v>22</v>
@@ -1745,7 +1745,7 @@
         <v>58</v>
       </c>
       <c r="C24" s="2">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="D24" s="2">
         <v>2.4</v>
@@ -1765,7 +1765,7 @@
         <v>60</v>
       </c>
       <c r="C25" s="2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D25" s="2">
         <v>15</v>
@@ -1785,7 +1785,7 @@
         <v>62</v>
       </c>
       <c r="C26" s="2">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D26" s="2">
         <v>17</v>
@@ -1805,7 +1805,7 @@
         <v>64</v>
       </c>
       <c r="C27" s="2">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D27" s="2">
         <v>22</v>
@@ -1825,7 +1825,7 @@
         <v>66</v>
       </c>
       <c r="C28" s="2">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D28" s="2">
         <v>23</v>
@@ -1868,7 +1868,7 @@
         <v>71</v>
       </c>
       <c r="C30" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D30" s="2">
         <v>18</v>
@@ -1888,7 +1888,7 @@
         <v>73</v>
       </c>
       <c r="C31" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D31" s="2">
         <v>35</v>
@@ -1908,7 +1908,7 @@
         <v>75</v>
       </c>
       <c r="C32" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D32" s="2">
         <v>8</v>
@@ -1928,7 +1928,7 @@
         <v>77</v>
       </c>
       <c r="C33" s="2">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D33" s="2">
         <v>25</v>
@@ -1948,7 +1948,7 @@
         <v>79</v>
       </c>
       <c r="C34" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D34" s="2">
         <v>24.5</v>
@@ -1968,7 +1968,7 @@
         <v>81</v>
       </c>
       <c r="C35" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D35" s="2">
         <v>28</v>
@@ -2111,7 +2111,7 @@
         <v>96</v>
       </c>
       <c r="C42" s="2">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D42" s="2">
         <v>18</v>
@@ -2131,7 +2131,7 @@
         <v>98</v>
       </c>
       <c r="C43" s="2">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D43" s="2">
         <v>15</v>
@@ -2154,7 +2154,7 @@
         <v>101</v>
       </c>
       <c r="C44" s="2">
-        <v>259</v>
+        <v>236</v>
       </c>
       <c r="D44" s="2">
         <v>1</v>
@@ -2174,7 +2174,7 @@
         <v>103</v>
       </c>
       <c r="C45" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D45" s="2">
         <v>6</v>
@@ -2194,7 +2194,7 @@
         <v>105</v>
       </c>
       <c r="C46" s="2">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D46" s="2">
         <v>2.8</v>
@@ -2217,7 +2217,7 @@
         <v>108</v>
       </c>
       <c r="C47" s="2">
-        <v>253</v>
+        <v>22</v>
       </c>
       <c r="D47" s="2">
         <v>2.4</v>

</xml_diff>

<commit_message>
Configure date & time.
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -358,9 +358,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -378,11 +378,40 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="0"/>
       <name val="Arial"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -395,9 +424,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -409,18 +445,41 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -433,14 +492,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -449,13 +508,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -471,58 +523,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
@@ -538,157 +538,169 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -701,18 +713,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -735,7 +735,18 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -745,7 +756,22 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -768,8 +794,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -785,32 +811,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -832,148 +832,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1290,7 +1290,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="2">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2">
         <v>6.5</v>
@@ -1310,7 +1310,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="2">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D3" s="2">
         <v>6.5</v>
@@ -1330,7 +1330,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="2">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D4" s="2">
         <v>6.5</v>
@@ -1350,7 +1350,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="2">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D5" s="2">
         <v>52</v>
@@ -1370,7 +1370,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="2">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D6" s="2">
         <v>99</v>
@@ -1390,7 +1390,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2">
         <v>102</v>
@@ -1410,7 +1410,7 @@
         <v>21</v>
       </c>
       <c r="C8" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" s="2">
         <v>24</v>
@@ -1430,7 +1430,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="2">
         <v>28</v>
@@ -1453,7 +1453,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D10" s="2">
         <v>79</v>
@@ -1473,7 +1473,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D11" s="2">
         <v>12.5</v>
@@ -1496,7 +1496,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="2">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D12" s="2">
         <v>128</v>
@@ -1516,7 +1516,7 @@
         <v>33</v>
       </c>
       <c r="C13" s="2">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D13" s="2">
         <v>112</v>
@@ -1556,7 +1556,7 @@
         <v>37</v>
       </c>
       <c r="C15" s="2">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D15" s="2">
         <v>34.5</v>
@@ -1576,7 +1576,7 @@
         <v>39</v>
       </c>
       <c r="C16" s="2">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="D16" s="2">
         <v>18</v>
@@ -1619,7 +1619,7 @@
         <v>44</v>
       </c>
       <c r="C18" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D18" s="2">
         <v>11</v>
@@ -1639,7 +1639,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="2">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2">
         <v>22</v>
@@ -1659,7 +1659,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D20" s="2">
         <v>9</v>
@@ -1679,7 +1679,7 @@
         <v>50</v>
       </c>
       <c r="C21" s="2">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D21" s="2">
         <v>15</v>
@@ -1699,7 +1699,7 @@
         <v>52</v>
       </c>
       <c r="C22" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D22" s="2">
         <v>15</v>
@@ -1725,7 +1725,7 @@
         <v>56</v>
       </c>
       <c r="C23" s="2">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D23" s="2">
         <v>22</v>
@@ -1765,7 +1765,7 @@
         <v>60</v>
       </c>
       <c r="C25" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D25" s="2">
         <v>15</v>
@@ -1805,7 +1805,7 @@
         <v>64</v>
       </c>
       <c r="C27" s="2">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D27" s="2">
         <v>22</v>
@@ -1825,7 +1825,7 @@
         <v>66</v>
       </c>
       <c r="C28" s="2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D28" s="2">
         <v>23</v>
@@ -1868,7 +1868,7 @@
         <v>71</v>
       </c>
       <c r="C30" s="2">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D30" s="2">
         <v>18</v>
@@ -1888,7 +1888,7 @@
         <v>73</v>
       </c>
       <c r="C31" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D31" s="2">
         <v>35</v>
@@ -1908,7 +1908,7 @@
         <v>75</v>
       </c>
       <c r="C32" s="2">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D32" s="2">
         <v>8</v>
@@ -1948,7 +1948,7 @@
         <v>79</v>
       </c>
       <c r="C34" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D34" s="2">
         <v>24.5</v>
@@ -1968,7 +1968,7 @@
         <v>81</v>
       </c>
       <c r="C35" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D35" s="2">
         <v>28</v>
@@ -2028,7 +2028,7 @@
         <v>87</v>
       </c>
       <c r="C38" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D38" s="2">
         <v>19</v>
@@ -2091,7 +2091,7 @@
         <v>94</v>
       </c>
       <c r="C41" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D41" s="2">
         <v>18</v>
@@ -2111,7 +2111,7 @@
         <v>96</v>
       </c>
       <c r="C42" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D42" s="2">
         <v>18</v>
@@ -2131,7 +2131,7 @@
         <v>98</v>
       </c>
       <c r="C43" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D43" s="2">
         <v>15</v>
@@ -2154,7 +2154,7 @@
         <v>101</v>
       </c>
       <c r="C44" s="2">
-        <v>236</v>
+        <v>281</v>
       </c>
       <c r="D44" s="2">
         <v>1</v>
@@ -2174,7 +2174,7 @@
         <v>103</v>
       </c>
       <c r="C45" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D45" s="2">
         <v>6</v>
@@ -2194,7 +2194,7 @@
         <v>105</v>
       </c>
       <c r="C46" s="2">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="D46" s="2">
         <v>2.8</v>
@@ -2217,7 +2217,7 @@
         <v>108</v>
       </c>
       <c r="C47" s="2">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D47" s="2">
         <v>2.4</v>
@@ -2240,7 +2240,7 @@
         <v>111</v>
       </c>
       <c r="C48">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E48" s="4">
         <v>2900</v>

</xml_diff>